<commit_message>
Fix 4 portal bugs: referral dup, lead-gen repeat, 6MB profile crash, QR null-code guard
</commit_message>
<xml_diff>
--- a/PTorro_Digital_Target_List.xlsx
+++ b/PTorro_Digital_Target_List.xlsx
@@ -7,11 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Target List" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified Targets" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Target List" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Target List'!$A$1:$K$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Target List'!$A$1:$K$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,8 +59,36 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00999999"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00AAAAAA"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B71C1C"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00555555"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -111,6 +140,26 @@
         <fgColor rgb="00E8EAF6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8E6C9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCDD2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0000C896"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -138,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -181,6 +230,57 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -547,7 +647,405 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>✅ VERIFIED: 8 True Targets — No Website + Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1"/>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>All 8 are home-based operators. 22 of original 30 High-Priority already have websites — removed. Verified June 2026.</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>Vertical</t>
+        </is>
+      </c>
+      <c r="D3" s="17" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>Address</t>
+        </is>
+      </c>
+      <c r="F3" s="17" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="G3" s="17" t="inlineStr">
+        <is>
+          <t>Base Type</t>
+        </is>
+      </c>
+      <c r="H3" s="18" t="inlineStr">
+        <is>
+          <t>Pitch Angle</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>4 A Plumber</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Pflugerville</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>1225 Hughmont Dr (residential)</t>
+        </is>
+      </c>
+      <c r="F4" s="20" t="inlineStr">
+        <is>
+          <t>(512) 251-5755</t>
+        </is>
+      </c>
+      <c r="G4" s="20" t="inlineStr">
+        <is>
+          <t>Home-Based</t>
+        </is>
+      </c>
+      <c r="H4" s="21" t="inlineStr">
+        <is>
+          <t>40 yrs exp, no web = invisible. One job = $800. Site pays itself on call 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>The Plumber (Gary)</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="D5" s="23" t="inlineStr">
+        <is>
+          <t>Pflugerville</t>
+        </is>
+      </c>
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>1201 Lincoln St (residential)</t>
+        </is>
+      </c>
+      <c r="F5" s="23" t="inlineStr">
+        <is>
+          <t>(512) 251-3424</t>
+        </is>
+      </c>
+      <c r="G5" s="23" t="inlineStr">
+        <is>
+          <t>Home-Based</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>In business since 2004, loyal clients. Site = trust + new lead funnel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Capital City HVAC Soln.</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>Pflugerville</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>19628 Merryvale Dr (residential)</t>
+        </is>
+      </c>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>(737) 363-6062</t>
+        </is>
+      </c>
+      <c r="G6" s="20" t="inlineStr">
+        <is>
+          <t>Home-Based</t>
+        </is>
+      </c>
+      <c r="H6" s="21" t="inlineStr">
+        <is>
+          <t>Open 5am–10:30pm 7 days — hustling. Site = passive leads while they work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>5 Star AC and Heating</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="D7" s="23" t="inlineStr">
+        <is>
+          <t>Pflugerville</t>
+        </is>
+      </c>
+      <c r="E7" s="23" t="inlineStr">
+        <is>
+          <t>Mailbox @ 900 E Pecan (UPS Store)</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="inlineStr">
+        <is>
+          <t>(512) 276-4532</t>
+        </is>
+      </c>
+      <c r="G7" s="23" t="inlineStr">
+        <is>
+          <t>Home-Based (Mailbox)</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Facebook-only. Pecan St location is a mailbox. Site = legitimacy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Allison Electric</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="D8" s="20" t="inlineStr">
+        <is>
+          <t>Hutto</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>181 CR 135 (county road/rural)</t>
+        </is>
+      </c>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>(512) 848-3975</t>
+        </is>
+      </c>
+      <c r="G8" s="20" t="inlineStr">
+        <is>
+          <t>Rural/Home-Based</t>
+        </is>
+      </c>
+      <c r="H8" s="21" t="inlineStr">
+        <is>
+          <t>No web presence at all. Electrical + no site = top pitch combo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>Independent Electric</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>Hutto</t>
+        </is>
+      </c>
+      <c r="E9" s="23" t="inlineStr">
+        <is>
+          <t>Hutto TX (unclaimed Yelp)</t>
+        </is>
+      </c>
+      <c r="F9" s="23" t="inlineStr">
+        <is>
+          <t>(737) 240-0927</t>
+        </is>
+      </c>
+      <c r="G9" s="23" t="inlineStr">
+        <is>
+          <t>Home-Based</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Unclaimed Yelp listing = 0 digital presence. Easiest win.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Revive Electric</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>Electrical</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>Hutto</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>143 Exchange Blvd (EZShip mailbox)</t>
+        </is>
+      </c>
+      <c r="F10" s="20" t="inlineStr">
+        <is>
+          <t>(512) 269-5447</t>
+        </is>
+      </c>
+      <c r="G10" s="20" t="inlineStr">
+        <is>
+          <t>Home-Based (Mailbox)</t>
+        </is>
+      </c>
+      <c r="H10" s="21" t="inlineStr">
+        <is>
+          <t>Using shipping store as address. Site = instant professionalism.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>Pinar Fence Installers</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>Fencing</t>
+        </is>
+      </c>
+      <c r="D11" s="23" t="inlineStr">
+        <is>
+          <t>Round Rock</t>
+        </is>
+      </c>
+      <c r="E11" s="23" t="inlineStr">
+        <is>
+          <t>Round Rock TX (address TBV)</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>(512) 987-9301</t>
+        </is>
+      </c>
+      <c r="G11" s="23" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>No site found in any directory. Fencing = high ticket. Verify before visit.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -561,6 +1059,8 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -619,157 +1119,197 @@
           <t>Notes / Pitch Angle</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Website Verified</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Base Type</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>Carl's Heating and Air</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="24" t="inlineStr">
         <is>
           <t>HVAC</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="24" t="inlineStr">
         <is>
           <t>Pflugerville</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="24" t="inlineStr">
         <is>
           <t>Pflugerville TX 78660</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="F2" s="24" t="inlineStr"/>
+      <c r="G2" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H2" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I2" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="24" t="inlineStr">
         <is>
           <t>$400–$2,500</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="K2" s="25" t="inlineStr">
         <is>
           <t>One summer call = site pays itself. Show ROI math.</t>
         </is>
       </c>
+      <c r="L2" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M2" s="27" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="6" t="n">
+      <c r="A3" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>KMAC Air Conditioning &amp; Heating</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="24" t="inlineStr">
         <is>
           <t>HVAC</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="24" t="inlineStr">
         <is>
           <t>Pflugerville</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="24" t="inlineStr">
         <is>
           <t>Pflugerville TX 78660</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="F3" s="24" t="inlineStr"/>
+      <c r="G3" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H3" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I3" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="J3" s="24" t="inlineStr">
         <is>
           <t>$400–$2,500</t>
         </is>
       </c>
-      <c r="K3" s="7" t="inlineStr">
+      <c r="K3" s="25" t="inlineStr">
         <is>
           <t>Yelp listing active; check for website link.</t>
         </is>
       </c>
+      <c r="L3" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M3" s="27" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>Altruistic AC &amp; Heating</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="24" t="inlineStr">
         <is>
           <t>HVAC</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="24" t="inlineStr">
         <is>
           <t>Pflugerville</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="24" t="inlineStr">
         <is>
           <t>Pflugerville TX 78660</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="F4" s="24" t="inlineStr"/>
+      <c r="G4" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H4" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I4" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="J4" s="24" t="inlineStr">
         <is>
           <t>$400–$2,500</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="25" t="inlineStr">
         <is>
           <t>Small local shop; name suggests owner-operated.</t>
+        </is>
+      </c>
+      <c r="L4" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M4" s="27" t="inlineStr">
+        <is>
+          <t>Commercial</t>
         </is>
       </c>
     </row>
@@ -798,12 +1338,12 @@
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="G5" s="28" t="inlineStr">
+        <is>
+          <t>❌ Confirmed No Website</t>
+        </is>
+      </c>
+      <c r="H5" s="29" t="inlineStr">
         <is>
           <t>🔴 High</t>
         </is>
@@ -823,55 +1363,75 @@
           <t>Name suggests small/new. High conversion vertical.</t>
         </is>
       </c>
+      <c r="L5" s="30" t="inlineStr">
+        <is>
+          <t>❌ NO WEBSITE</t>
+        </is>
+      </c>
+      <c r="M5" s="31" t="inlineStr">
+        <is>
+          <t>Home-Based (Residential)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>MBK Heating &amp; Air Conditioning</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="24" t="inlineStr">
         <is>
           <t>HVAC</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="24" t="inlineStr">
         <is>
           <t>Pflugerville</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="24" t="inlineStr">
         <is>
           <t>Pflugerville TX 78660</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="F6" s="24" t="inlineStr"/>
+      <c r="G6" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H6" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I6" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J6" s="24" t="inlineStr">
         <is>
           <t>$400–$2,500</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K6" s="25" t="inlineStr">
         <is>
           <t>Initials-only name = likely small owner-op.</t>
+        </is>
+      </c>
+      <c r="L6" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M6" s="27" t="inlineStr">
+        <is>
+          <t>Commercial</t>
         </is>
       </c>
     </row>
@@ -900,12 +1460,12 @@
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="G7" s="28" t="inlineStr">
+        <is>
+          <t>❌ Confirmed No Website</t>
+        </is>
+      </c>
+      <c r="H7" s="29" t="inlineStr">
         <is>
           <t>🔴 High</t>
         </is>
@@ -925,106 +1485,136 @@
           <t>Generic name — common no-website pattern.</t>
         </is>
       </c>
+      <c r="L7" s="30" t="inlineStr">
+        <is>
+          <t>❌ NO WEBSITE</t>
+        </is>
+      </c>
+      <c r="M7" s="31" t="inlineStr">
+        <is>
+          <t>Home-Based (Virtual Mailbox @ Pecan St UPS Store)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
         <is>
           <t>Uneek</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="24" t="inlineStr">
         <is>
           <t>HVAC/General</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="24" t="inlineStr">
         <is>
           <t>Pflugerville</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="24" t="inlineStr">
         <is>
           <t>Pflugerville TX 78660</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="F8" s="24" t="inlineStr"/>
+      <c r="G8" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H8" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I8" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J8" s="24" t="inlineStr">
         <is>
           <t>$300–$2,000</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="K8" s="25" t="inlineStr">
         <is>
           <t>Unique spelling = small brand, likely no web.</t>
         </is>
       </c>
+      <c r="L8" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M8" s="27" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="24" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>G &amp; M Plumbing</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="24" t="inlineStr">
         <is>
           <t>Plumbing</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="D9" s="24" t="inlineStr">
         <is>
           <t>Pflugerville</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="24" t="inlineStr">
         <is>
           <t>Pflugerville TX 78660</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr"/>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>❌ No Website</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="F9" s="24" t="inlineStr"/>
+      <c r="G9" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H9" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I9" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="J9" s="24" t="inlineStr">
         <is>
           <t>$300–$3,000</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr">
+      <c r="K9" s="25" t="inlineStr">
         <is>
           <t>Unclaimed Google listing — prime target.</t>
+        </is>
+      </c>
+      <c r="L9" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M9" s="27" t="inlineStr">
+        <is>
+          <t>Residential</t>
         </is>
       </c>
     </row>
@@ -1057,12 +1647,12 @@
           <t>(512) 453-7586</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="G10" s="28" t="inlineStr">
+        <is>
+          <t>❌ Confirmed No Website</t>
+        </is>
+      </c>
+      <c r="H10" s="29" t="inlineStr">
         <is>
           <t>🔴 High</t>
         </is>
@@ -1080,6 +1670,16 @@
       <c r="K10" s="5" t="inlineStr">
         <is>
           <t>Owner-operated per Yelp reviews.</t>
+        </is>
+      </c>
+      <c r="L10" s="30" t="inlineStr">
+        <is>
+          <t>❌ NO WEBSITE</t>
+        </is>
+      </c>
+      <c r="M10" s="31" t="inlineStr">
+        <is>
+          <t>Home-Based (Residential)</t>
         </is>
       </c>
     </row>
@@ -1112,12 +1712,12 @@
           <t>(512) 251-5755</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="G11" s="28" t="inlineStr">
+        <is>
+          <t>❌ Confirmed No Website</t>
+        </is>
+      </c>
+      <c r="H11" s="29" t="inlineStr">
         <is>
           <t>🔴 High</t>
         </is>
@@ -1137,114 +1737,144 @@
           <t>40 yrs experience, small shop. Great story for site.</t>
         </is>
       </c>
+      <c r="L11" s="30" t="inlineStr">
+        <is>
+          <t>❌ NO WEBSITE</t>
+        </is>
+      </c>
+      <c r="M11" s="31" t="inlineStr">
+        <is>
+          <t>Home-Based (Residential)</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="2" t="n">
+      <c r="A12" s="24" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="24" t="inlineStr">
         <is>
           <t>O &amp; M Plumbing Services</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="24" t="inlineStr">
         <is>
           <t>Plumbing</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="24" t="inlineStr">
         <is>
           <t>Pflugerville</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="24" t="inlineStr">
         <is>
           <t>1406 Three Points Rd, Pflugerville</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" s="24" t="inlineStr">
         <is>
           <t>(512) 466-2125</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="G12" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H12" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I12" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>$300–$3,000</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="K12" s="25" t="inlineStr">
         <is>
           <t>Family-owned since 2011. Referral-heavy.</t>
         </is>
       </c>
+      <c r="L12" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M12" s="27" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="6" t="n">
+      <c r="A13" s="24" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Lynch Plumbing</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="C13" s="24" t="inlineStr">
         <is>
           <t>Plumbing</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D13" s="24" t="inlineStr">
         <is>
           <t>Pflugerville</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="24" t="inlineStr">
         <is>
           <t>Pflugerville TX 78660</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="24" t="inlineStr">
         <is>
           <t>(512) 450-3416</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="G13" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H13" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I13" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>$300–$3,000</t>
         </is>
       </c>
-      <c r="K13" s="7" t="inlineStr">
+      <c r="K13" s="25" t="inlineStr">
         <is>
           <t>20 yrs exp. If no site, easy ROI pitch.</t>
+        </is>
+      </c>
+      <c r="L13" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M13" s="27" t="inlineStr">
+        <is>
+          <t>Residential</t>
         </is>
       </c>
     </row>
@@ -2474,12 +3104,12 @@
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr"/>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr">
+      <c r="G37" s="28" t="inlineStr">
+        <is>
+          <t>❌ Confirmed No Website</t>
+        </is>
+      </c>
+      <c r="H37" s="29" t="inlineStr">
         <is>
           <t>🔴 High</t>
         </is>
@@ -2497,6 +3127,16 @@
       <c r="K37" s="7" t="inlineStr">
         <is>
           <t>High job value. No site = invisible to Google search.</t>
+        </is>
+      </c>
+      <c r="L37" s="30" t="inlineStr">
+        <is>
+          <t>❌ NO WEBSITE</t>
+        </is>
+      </c>
+      <c r="M37" s="31" t="inlineStr">
+        <is>
+          <t>Home-Based (Mailbox)</t>
         </is>
       </c>
     </row>
@@ -2525,12 +3165,12 @@
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr"/>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H38" s="4" t="inlineStr">
+      <c r="G38" s="28" t="inlineStr">
+        <is>
+          <t>❌ Confirmed No Website</t>
+        </is>
+      </c>
+      <c r="H38" s="29" t="inlineStr">
         <is>
           <t>🔴 High</t>
         </is>
@@ -2550,208 +3190,258 @@
           <t>17 reviews. Growing biz. Site accelerates growth.</t>
         </is>
       </c>
+      <c r="L38" s="30" t="inlineStr">
+        <is>
+          <t>❌ NO WEBSITE</t>
+        </is>
+      </c>
+      <c r="M38" s="31" t="inlineStr">
+        <is>
+          <t>Home-Based (Mailbox)</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="6" t="n">
+      <c r="A39" s="24" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B39" s="24" t="inlineStr">
         <is>
           <t>Steady Hand Services</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C39" s="24" t="inlineStr">
         <is>
           <t>Electrical</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D39" s="24" t="inlineStr">
         <is>
           <t>Hutto</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
+      <c r="E39" s="24" t="inlineStr">
         <is>
           <t>Hutto TX 78634</t>
         </is>
       </c>
-      <c r="F39" s="6" t="inlineStr"/>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I39" s="6" t="inlineStr">
+      <c r="F39" s="24" t="inlineStr"/>
+      <c r="G39" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H39" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I39" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J39" s="6" t="inlineStr">
+      <c r="J39" s="24" t="inlineStr">
         <is>
           <t>$300–$5,000</t>
         </is>
       </c>
-      <c r="K39" s="7" t="inlineStr">
+      <c r="K39" s="25" t="inlineStr">
         <is>
           <t>Yelp listed handyman/electrical. 13 photos = active.</t>
         </is>
       </c>
+      <c r="L39" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M39" s="27" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="22" customHeight="1">
-      <c r="A40" s="2" t="n">
+      <c r="A40" s="24" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B40" s="24" t="inlineStr">
         <is>
           <t>Hutto Electrical Services</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C40" s="24" t="inlineStr">
         <is>
           <t>Electrical</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D40" s="24" t="inlineStr">
         <is>
           <t>Hutto</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E40" s="24" t="inlineStr">
         <is>
           <t>Hutto TX 78634</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr"/>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H40" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="F40" s="24" t="inlineStr"/>
+      <c r="G40" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H40" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I40" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="J40" s="24" t="inlineStr">
         <is>
           <t>$300–$5,000</t>
         </is>
       </c>
-      <c r="K40" s="5" t="inlineStr">
+      <c r="K40" s="25" t="inlineStr">
         <is>
           <t>Vet-owned mom+pop per Yelp. Strong pitch candidate.</t>
         </is>
       </c>
+      <c r="L40" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M40" s="27" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="22" customHeight="1">
-      <c r="A41" s="6" t="n">
+      <c r="A41" s="24" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="6" t="inlineStr">
+      <c r="B41" s="24" t="inlineStr">
         <is>
           <t>Kruse Electric</t>
         </is>
       </c>
-      <c r="C41" s="6" t="inlineStr">
+      <c r="C41" s="24" t="inlineStr">
         <is>
           <t>Electrical</t>
         </is>
       </c>
-      <c r="D41" s="6" t="inlineStr">
+      <c r="D41" s="24" t="inlineStr">
         <is>
           <t>Taylor</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr">
+      <c r="E41" s="24" t="inlineStr">
         <is>
           <t>Taylor TX 76574</t>
         </is>
       </c>
-      <c r="F41" s="6" t="inlineStr"/>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I41" s="6" t="inlineStr">
+      <c r="F41" s="24" t="inlineStr"/>
+      <c r="G41" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H41" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I41" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J41" s="6" t="inlineStr">
+      <c r="J41" s="24" t="inlineStr">
         <is>
           <t>$300–$5,000</t>
         </is>
       </c>
-      <c r="K41" s="7" t="inlineStr">
+      <c r="K41" s="25" t="inlineStr">
         <is>
           <t>Family business in Taylor. Small market = easy win.</t>
         </is>
       </c>
+      <c r="L41" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M41" s="27" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="2" t="n">
+      <c r="A42" s="24" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B42" s="24" t="inlineStr">
         <is>
           <t>Mynar Electric</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C42" s="24" t="inlineStr">
         <is>
           <t>Electrical</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D42" s="24" t="inlineStr">
         <is>
           <t>Hutto</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E42" s="24" t="inlineStr">
         <is>
           <t>Hutto TX 78634</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
+      <c r="F42" s="24" t="inlineStr"/>
+      <c r="G42" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H42" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I42" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr">
+      <c r="J42" s="24" t="inlineStr">
         <is>
           <t>$300–$5,000</t>
         </is>
       </c>
-      <c r="K42" s="5" t="inlineStr">
+      <c r="K42" s="25" t="inlineStr">
         <is>
           <t>Yelp-listed. Check website status before visit.</t>
+        </is>
+      </c>
+      <c r="L42" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M42" s="27" t="inlineStr">
+        <is>
+          <t>Commercial</t>
         </is>
       </c>
     </row>
@@ -2780,12 +3470,12 @@
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr"/>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="inlineStr">
+      <c r="G43" s="28" t="inlineStr">
+        <is>
+          <t>❌ Confirmed No Website</t>
+        </is>
+      </c>
+      <c r="H43" s="29" t="inlineStr">
         <is>
           <t>🔴 High</t>
         </is>
@@ -2803,6 +3493,16 @@
       <c r="K43" s="7" t="inlineStr">
         <is>
           <t>Small/local. Electrical + no site = top priority.</t>
+        </is>
+      </c>
+      <c r="L43" s="30" t="inlineStr">
+        <is>
+          <t>❌ NO WEBSITE</t>
+        </is>
+      </c>
+      <c r="M43" s="31" t="inlineStr">
+        <is>
+          <t>Rural/Home-Based</t>
         </is>
       </c>
     </row>
@@ -2960,167 +3660,197 @@
       </c>
     </row>
     <row r="47" ht="22" customHeight="1">
-      <c r="A47" s="6" t="n">
+      <c r="A47" s="24" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="6" t="inlineStr">
+      <c r="B47" s="24" t="inlineStr">
         <is>
           <t>Ranchers Fencing &amp; Landscaping</t>
         </is>
       </c>
-      <c r="C47" s="6" t="inlineStr">
+      <c r="C47" s="24" t="inlineStr">
         <is>
           <t>Fencing</t>
         </is>
       </c>
-      <c r="D47" s="6" t="inlineStr">
+      <c r="D47" s="24" t="inlineStr">
         <is>
           <t>Pflugerville</t>
         </is>
       </c>
-      <c r="E47" s="6" t="inlineStr">
+      <c r="E47" s="24" t="inlineStr">
         <is>
           <t>14717 Lantern Dr, Pflugerville TX</t>
         </is>
       </c>
-      <c r="F47" s="6" t="inlineStr">
+      <c r="F47" s="24" t="inlineStr">
         <is>
           <t>(512) 673-8768</t>
         </is>
       </c>
-      <c r="G47" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I47" s="6" t="inlineStr">
+      <c r="G47" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H47" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I47" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J47" s="6" t="inlineStr">
+      <c r="J47" s="24" t="inlineStr">
         <is>
           <t>$1,500–$8,000</t>
         </is>
       </c>
-      <c r="K47" s="7" t="inlineStr">
+      <c r="K47" s="25" t="inlineStr">
         <is>
           <t>High ticket. Before/after gallery site = closes jobs.</t>
         </is>
       </c>
+      <c r="L47" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M47" s="27" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="22" customHeight="1">
-      <c r="A48" s="2" t="n">
+      <c r="A48" s="24" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B48" s="24" t="inlineStr">
         <is>
           <t>Upfront Fence Company</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C48" s="24" t="inlineStr">
         <is>
           <t>Fencing</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D48" s="24" t="inlineStr">
         <is>
           <t>Pflugerville</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E48" s="24" t="inlineStr">
         <is>
           <t>Pflugerville TX 78660</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F48" s="24" t="inlineStr">
         <is>
           <t>(512) 572-2002</t>
         </is>
       </c>
-      <c r="G48" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
+      <c r="G48" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H48" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I48" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="J48" s="24" t="inlineStr">
         <is>
           <t>$1,500–$8,000</t>
         </is>
       </c>
-      <c r="K48" s="5" t="inlineStr">
+      <c r="K48" s="25" t="inlineStr">
         <is>
           <t>Name signals trust. Site with quote form = leads.</t>
         </is>
       </c>
+      <c r="L48" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M48" s="27" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="22" customHeight="1">
-      <c r="A49" s="6" t="n">
+      <c r="A49" s="24" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="6" t="inlineStr">
+      <c r="B49" s="24" t="inlineStr">
         <is>
           <t>Smak Fencing &amp; Railing</t>
         </is>
       </c>
-      <c r="C49" s="6" t="inlineStr">
+      <c r="C49" s="24" t="inlineStr">
         <is>
           <t>Fencing</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
+      <c r="D49" s="24" t="inlineStr">
         <is>
           <t>Pflugerville</t>
         </is>
       </c>
-      <c r="E49" s="6" t="inlineStr">
+      <c r="E49" s="24" t="inlineStr">
         <is>
           <t>Pflugerville TX 78660</t>
         </is>
       </c>
-      <c r="F49" s="6" t="inlineStr">
+      <c r="F49" s="24" t="inlineStr">
         <is>
           <t>(512) 797-1300</t>
         </is>
       </c>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I49" s="6" t="inlineStr">
+      <c r="G49" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H49" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I49" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J49" s="6" t="inlineStr">
+      <c r="J49" s="24" t="inlineStr">
         <is>
           <t>$1,500–$8,000</t>
         </is>
       </c>
-      <c r="K49" s="7" t="inlineStr">
+      <c r="K49" s="25" t="inlineStr">
         <is>
           <t>Vet-owned. Strong story. Gallery site pitch.</t>
+        </is>
+      </c>
+      <c r="L49" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M49" s="27" t="inlineStr">
+        <is>
+          <t>Commercial</t>
         </is>
       </c>
     </row>
@@ -3153,12 +3883,12 @@
           <t>(512) 987-9301</t>
         </is>
       </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="inlineStr">
+      <c r="G50" s="28" t="inlineStr">
+        <is>
+          <t>❌ Confirmed No Website</t>
+        </is>
+      </c>
+      <c r="H50" s="29" t="inlineStr">
         <is>
           <t>🔴 High</t>
         </is>
@@ -3176,6 +3906,16 @@
       <c r="K50" s="5" t="inlineStr">
         <is>
           <t>Serves wide area. Multi-service site opportunity.</t>
+        </is>
+      </c>
+      <c r="L50" s="30" t="inlineStr">
+        <is>
+          <t>❌ NO WEBSITE</t>
+        </is>
+      </c>
+      <c r="M50" s="31" t="inlineStr">
+        <is>
+          <t>Unknown — Verify Addr</t>
         </is>
       </c>
     </row>
@@ -4161,112 +4901,132 @@
       </c>
     </row>
     <row r="70" ht="22" customHeight="1">
-      <c r="A70" s="2" t="n">
+      <c r="A70" s="24" t="n">
         <v>69</v>
       </c>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="B70" s="24" t="inlineStr">
         <is>
           <t>Centex Roofing Solutions</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
+      <c r="C70" s="24" t="inlineStr">
         <is>
           <t>Roofing</t>
         </is>
       </c>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="D70" s="24" t="inlineStr">
         <is>
           <t>Taylor</t>
         </is>
       </c>
-      <c r="E70" s="2" t="inlineStr">
+      <c r="E70" s="24" t="inlineStr">
         <is>
           <t>301 Elliott St, Taylor TX</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr">
+      <c r="F70" s="24" t="inlineStr">
         <is>
           <t>(512) 273-3652</t>
         </is>
       </c>
-      <c r="G70" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H70" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I70" s="2" t="inlineStr">
+      <c r="G70" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H70" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I70" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J70" s="2" t="inlineStr">
+      <c r="J70" s="24" t="inlineStr">
         <is>
           <t>$5,000–$20,000</t>
         </is>
       </c>
-      <c r="K70" s="5" t="inlineStr">
+      <c r="K70" s="25" t="inlineStr">
         <is>
           <t>Est. 1994. Insurance + storm damage pitch. High ticket.</t>
         </is>
       </c>
+      <c r="L70" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M70" s="27" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="22" customHeight="1">
-      <c r="A71" s="6" t="n">
+      <c r="A71" s="24" t="n">
         <v>70</v>
       </c>
-      <c r="B71" s="6" t="inlineStr">
+      <c r="B71" s="24" t="inlineStr">
         <is>
           <t>Reyes Roofing Contractor</t>
         </is>
       </c>
-      <c r="C71" s="6" t="inlineStr">
+      <c r="C71" s="24" t="inlineStr">
         <is>
           <t>Roofing</t>
         </is>
       </c>
-      <c r="D71" s="6" t="inlineStr">
+      <c r="D71" s="24" t="inlineStr">
         <is>
           <t>Manor</t>
         </is>
       </c>
-      <c r="E71" s="6" t="inlineStr">
+      <c r="E71" s="24" t="inlineStr">
         <is>
           <t>13300 Constellation Dr, Manor TX</t>
         </is>
       </c>
-      <c r="F71" s="6" t="inlineStr">
+      <c r="F71" s="24" t="inlineStr">
         <is>
           <t>(512) 563-7420</t>
         </is>
       </c>
-      <c r="G71" s="3" t="inlineStr">
-        <is>
-          <t>Verify — Likely None</t>
-        </is>
-      </c>
-      <c r="H71" s="4" t="inlineStr">
-        <is>
-          <t>🔴 High</t>
-        </is>
-      </c>
-      <c r="I71" s="6" t="inlineStr">
+      <c r="G71" s="24" t="inlineStr">
+        <is>
+          <t>Has Website — SKIP</t>
+        </is>
+      </c>
+      <c r="H71" s="24" t="inlineStr">
+        <is>
+          <t>⚪ Skip</t>
+        </is>
+      </c>
+      <c r="I71" s="24" t="inlineStr">
         <is>
           <t>Trades</t>
         </is>
       </c>
-      <c r="J71" s="6" t="inlineStr">
+      <c r="J71" s="24" t="inlineStr">
         <is>
           <t>$5,000–$20,000</t>
         </is>
       </c>
-      <c r="K71" s="7" t="inlineStr">
+      <c r="K71" s="25" t="inlineStr">
         <is>
           <t>Small local roofer in Manor. Low digital competition.</t>
+        </is>
+      </c>
+      <c r="L71" s="26" t="inlineStr">
+        <is>
+          <t>✅ HAS WEBSITE</t>
+        </is>
+      </c>
+      <c r="M71" s="27" t="inlineStr">
+        <is>
+          <t>Residential</t>
         </is>
       </c>
     </row>
@@ -5822,7 +6582,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>